<commit_message>
Add GEX logo to tear sheet header
Copies assets/gex_logo.png into the repo and inserts it via
xlsxwriter insert_image into the top-right corner of the header,
replacing the 'GEX ×' text placeholder. Logo scales to ~70px tall
and floats over the date + fund-name rows.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Tear_Sheet_Feb2026.xlsx
+++ b/output/Tear_Sheet_Feb2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="113">
   <si>
     <t>Date</t>
   </si>
@@ -159,9 +159,6 @@
   </si>
   <si>
     <t>February 2026</t>
-  </si>
-  <si>
-    <t>GEX ×</t>
   </si>
   <si>
     <t>GREEN RENEWABLE STORAGE ENERGY MARKET</t>
@@ -366,7 +363,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -382,9 +379,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FF2E7D32"/>
+      <sz val="9"/>
+      <color rgb="FF1A1A1A"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -408,13 +404,6 @@
       <b/>
       <sz val="10"/>
       <color rgb="FF2E7D32"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF1A1A1A"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -620,13 +609,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -642,10 +631,10 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -653,46 +642,43 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="15" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="15" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1631,6 +1617,44 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>97571</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>69861</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="gex_logo.png"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6334125" y="19050"/>
+          <a:ext cx="230921" cy="222261"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>26</xdr:row>
@@ -1644,7 +1668,7 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvPr id="3" name="Chart 2"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1653,7 +1677,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1674,7 +1698,7 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvPr id="4" name="Chart 3"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -1683,7 +1707,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2650,9 +2674,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-      <c r="J1" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
@@ -2662,7 +2684,7 @@
     </row>
     <row r="2" spans="1:17" ht="26" customHeight="1">
       <c r="B2" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -2681,7 +2703,7 @@
     </row>
     <row r="3" spans="1:17" ht="26" customHeight="1">
       <c r="B3" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -2720,7 +2742,7 @@
     <row r="5" spans="1:17" ht="8" customHeight="1"/>
     <row r="6" spans="1:17" ht="17" customHeight="1">
       <c r="B6" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5"/>
@@ -2730,7 +2752,7 @@
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
@@ -2740,122 +2762,122 @@
       <c r="P6" s="5"/>
     </row>
     <row r="7" spans="1:17">
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="7" t="s">
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+    </row>
+    <row r="8" spans="1:17">
+      <c r="B8" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="7"/>
-    </row>
-    <row r="8" spans="1:17">
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+    </row>
+    <row r="9" spans="1:17">
+      <c r="B9" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-    </row>
-    <row r="9" spans="1:17">
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+    </row>
+    <row r="10" spans="1:17">
+      <c r="B10" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
-    </row>
-    <row r="10" spans="1:17">
-      <c r="B10" s="6" t="s">
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+      <c r="P10" s="2"/>
+    </row>
+    <row r="11" spans="1:17">
+      <c r="B11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
-      <c r="P10" s="6"/>
-    </row>
-    <row r="11" spans="1:17">
-      <c r="B11" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
     </row>
     <row r="12" spans="1:17" ht="10" customHeight="1">
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+      <c r="P12" s="2"/>
     </row>
     <row r="13" spans="1:17" ht="17" customHeight="1">
       <c r="B13" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C13" s="5"/>
       <c r="D13" s="5"/>
@@ -2865,7 +2887,7 @@
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
       <c r="J13" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
@@ -2875,127 +2897,127 @@
       <c r="P13" s="5"/>
     </row>
     <row r="14" spans="1:17" ht="12" customHeight="1">
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="9" t="s">
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="9" t="s">
+      <c r="P14" s="8"/>
+    </row>
+    <row r="15" spans="1:17" ht="26" customHeight="1">
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="P14" s="9"/>
-    </row>
-    <row r="15" spans="1:17" ht="26" customHeight="1">
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="10" t="s">
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
-      <c r="O15" s="10" t="s">
+      <c r="P15" s="9"/>
+    </row>
+    <row r="16" spans="1:17" ht="12" customHeight="1">
+      <c r="B16" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P15" s="10"/>
-    </row>
-    <row r="16" spans="1:17" ht="12" customHeight="1">
-      <c r="B16" s="11" t="s">
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="9" t="s">
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+      <c r="O16" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
-      <c r="O16" s="9" t="s">
+      <c r="P16" s="8"/>
+    </row>
+    <row r="17" spans="2:16" ht="26" customHeight="1">
+      <c r="B17" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="P16" s="9"/>
-    </row>
-    <row r="17" spans="2:16" ht="26" customHeight="1">
-      <c r="B17" s="11" t="s">
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="12" t="s">
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="11"/>
+      <c r="N17" s="11"/>
+      <c r="O17" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="K17" s="12"/>
-      <c r="L17" s="12"/>
-      <c r="M17" s="12"/>
-      <c r="N17" s="12"/>
-      <c r="O17" s="10" t="s">
+      <c r="P17" s="9"/>
+    </row>
+    <row r="18" spans="2:16" ht="10" customHeight="1">
+      <c r="B18" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="P17" s="10"/>
-    </row>
-    <row r="18" spans="2:16" ht="10" customHeight="1">
-      <c r="B18" s="11" t="s">
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
+      <c r="P18" s="2"/>
+    </row>
+    <row r="19" spans="2:16" ht="17" customHeight="1">
+      <c r="B19" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="6"/>
-      <c r="N18" s="6"/>
-      <c r="O18" s="6"/>
-      <c r="P18" s="6"/>
-    </row>
-    <row r="19" spans="2:16" ht="17" customHeight="1">
-      <c r="B19" s="11" t="s">
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="5" t="s">
-        <v>74</v>
       </c>
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
@@ -3005,136 +3027,136 @@
       <c r="P19" s="5"/>
     </row>
     <row r="20" spans="2:16">
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="13" t="s">
+      <c r="K20" s="12"/>
+      <c r="L20" s="12"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="K20" s="13"/>
-      <c r="L20" s="13"/>
-      <c r="M20" s="13"/>
-      <c r="N20" s="13"/>
-      <c r="O20" s="14" t="s">
+      <c r="P20" s="13"/>
+    </row>
+    <row r="21" spans="2:16">
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="P20" s="14"/>
-    </row>
-    <row r="21" spans="2:16">
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="13" t="s">
+      <c r="K21" s="12"/>
+      <c r="L21" s="12"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="12"/>
+      <c r="O21" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="K21" s="13"/>
-      <c r="L21" s="13"/>
-      <c r="M21" s="13"/>
-      <c r="N21" s="13"/>
-      <c r="O21" s="14" t="s">
+      <c r="P21" s="13"/>
+    </row>
+    <row r="22" spans="2:16">
+      <c r="B22" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="P21" s="14"/>
-    </row>
-    <row r="22" spans="2:16">
-      <c r="B22" s="11" t="s">
+      <c r="C22" s="10"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="10"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="13" t="s">
+      <c r="K22" s="12"/>
+      <c r="L22" s="12"/>
+      <c r="M22" s="12"/>
+      <c r="N22" s="12"/>
+      <c r="O22" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="K22" s="13"/>
-      <c r="L22" s="13"/>
-      <c r="M22" s="13"/>
-      <c r="N22" s="13"/>
-      <c r="O22" s="14" t="s">
+      <c r="P22" s="13"/>
+    </row>
+    <row r="23" spans="2:16">
+      <c r="B23" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="P22" s="14"/>
-    </row>
-    <row r="23" spans="2:16">
-      <c r="B23" s="11" t="s">
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="13" t="s">
+      <c r="K23" s="12"/>
+      <c r="L23" s="12"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="13"/>
-      <c r="O23" s="14" t="s">
+      <c r="P23" s="13"/>
+    </row>
+    <row r="24" spans="2:16">
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="P23" s="14"/>
-    </row>
-    <row r="24" spans="2:16">
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="13" t="s">
+      <c r="K24" s="12"/>
+      <c r="L24" s="12"/>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="K24" s="13"/>
-      <c r="L24" s="13"/>
-      <c r="M24" s="13"/>
-      <c r="N24" s="13"/>
-      <c r="O24" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="P24" s="14"/>
+      <c r="P24" s="13"/>
     </row>
     <row r="25" spans="2:16" ht="10" customHeight="1">
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
-      <c r="K25" s="6"/>
-      <c r="L25" s="6"/>
-      <c r="M25" s="6"/>
-      <c r="N25" s="6"/>
-      <c r="O25" s="6"/>
-      <c r="P25" s="6"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
+      <c r="L25" s="2"/>
+      <c r="M25" s="2"/>
+      <c r="N25" s="2"/>
+      <c r="O25" s="2"/>
+      <c r="P25" s="2"/>
     </row>
     <row r="26" spans="2:16" ht="17" customHeight="1">
       <c r="B26" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
@@ -3144,7 +3166,7 @@
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
       <c r="J26" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
@@ -3154,246 +3176,246 @@
       <c r="P26" s="5"/>
     </row>
     <row r="27" spans="2:16">
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="6"/>
-      <c r="J27" s="13" t="s">
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="K27" s="12"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="12"/>
+      <c r="N27" s="12"/>
+      <c r="O27" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="P27" s="14"/>
+    </row>
+    <row r="28" spans="2:16">
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="K27" s="13"/>
-      <c r="L27" s="13"/>
-      <c r="M27" s="13"/>
-      <c r="N27" s="13"/>
-      <c r="O27" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="P27" s="15"/>
-    </row>
-    <row r="28" spans="2:16">
-      <c r="B28" s="6"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6"/>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
-      <c r="I28" s="6"/>
-      <c r="J28" s="13" t="s">
+      <c r="K28" s="12"/>
+      <c r="L28" s="12"/>
+      <c r="M28" s="12"/>
+      <c r="N28" s="12"/>
+      <c r="O28" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="K28" s="13"/>
-      <c r="L28" s="13"/>
-      <c r="M28" s="13"/>
-      <c r="N28" s="13"/>
-      <c r="O28" s="15" t="s">
+      <c r="P28" s="14"/>
+    </row>
+    <row r="29" spans="2:16">
+      <c r="B29" s="2"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="P28" s="15"/>
-    </row>
-    <row r="29" spans="2:16">
-      <c r="B29" s="6"/>
-      <c r="C29" s="6"/>
-      <c r="D29" s="6"/>
-      <c r="E29" s="6"/>
-      <c r="F29" s="6"/>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6"/>
-      <c r="I29" s="6"/>
-      <c r="J29" s="13" t="s">
+      <c r="K29" s="12"/>
+      <c r="L29" s="12"/>
+      <c r="M29" s="12"/>
+      <c r="N29" s="12"/>
+      <c r="O29" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="K29" s="13"/>
-      <c r="L29" s="13"/>
-      <c r="M29" s="13"/>
-      <c r="N29" s="13"/>
-      <c r="O29" s="15" t="s">
+      <c r="P29" s="14"/>
+    </row>
+    <row r="30" spans="2:16">
+      <c r="B30" s="2"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="P29" s="15"/>
-    </row>
-    <row r="30" spans="2:16">
-      <c r="B30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="6"/>
-      <c r="J30" s="13" t="s">
+      <c r="K30" s="12"/>
+      <c r="L30" s="12"/>
+      <c r="M30" s="12"/>
+      <c r="N30" s="12"/>
+      <c r="O30" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="K30" s="13"/>
-      <c r="L30" s="13"/>
-      <c r="M30" s="13"/>
-      <c r="N30" s="13"/>
-      <c r="O30" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="P30" s="15"/>
+      <c r="P30" s="14"/>
     </row>
     <row r="31" spans="2:16">
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6"/>
-      <c r="I31" s="6"/>
-      <c r="J31" s="6"/>
-      <c r="K31" s="6"/>
-      <c r="L31" s="6"/>
-      <c r="M31" s="6"/>
-      <c r="N31" s="6"/>
-      <c r="O31" s="6"/>
-      <c r="P31" s="6"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
+      <c r="L31" s="2"/>
+      <c r="M31" s="2"/>
+      <c r="N31" s="2"/>
+      <c r="O31" s="2"/>
+      <c r="P31" s="2"/>
     </row>
     <row r="32" spans="2:16">
-      <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="6"/>
-      <c r="I32" s="6"/>
-      <c r="J32" s="6"/>
-      <c r="K32" s="6"/>
-      <c r="L32" s="6"/>
-      <c r="M32" s="6"/>
-      <c r="N32" s="6"/>
-      <c r="O32" s="6"/>
-      <c r="P32" s="6"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+      <c r="L32" s="2"/>
+      <c r="M32" s="2"/>
+      <c r="N32" s="2"/>
+      <c r="O32" s="2"/>
+      <c r="P32" s="2"/>
     </row>
     <row r="33" spans="2:16">
-      <c r="B33" s="6"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6"/>
-      <c r="I33" s="6"/>
-      <c r="J33" s="6"/>
-      <c r="K33" s="6"/>
-      <c r="L33" s="6"/>
-      <c r="M33" s="6"/>
-      <c r="N33" s="6"/>
-      <c r="O33" s="6"/>
-      <c r="P33" s="6"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
+      <c r="L33" s="2"/>
+      <c r="M33" s="2"/>
+      <c r="N33" s="2"/>
+      <c r="O33" s="2"/>
+      <c r="P33" s="2"/>
     </row>
     <row r="34" spans="2:16">
-      <c r="B34" s="6"/>
-      <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
-      <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="6"/>
-      <c r="K34" s="6"/>
-      <c r="L34" s="6"/>
-      <c r="M34" s="6"/>
-      <c r="N34" s="6"/>
-      <c r="O34" s="6"/>
-      <c r="P34" s="6"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
+      <c r="L34" s="2"/>
+      <c r="M34" s="2"/>
+      <c r="N34" s="2"/>
+      <c r="O34" s="2"/>
+      <c r="P34" s="2"/>
     </row>
     <row r="35" spans="2:16">
-      <c r="B35" s="6"/>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
-      <c r="H35" s="6"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="6"/>
-      <c r="K35" s="6"/>
-      <c r="L35" s="6"/>
-      <c r="M35" s="6"/>
-      <c r="N35" s="6"/>
-      <c r="O35" s="6"/>
-      <c r="P35" s="6"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
+      <c r="L35" s="2"/>
+      <c r="M35" s="2"/>
+      <c r="N35" s="2"/>
+      <c r="O35" s="2"/>
+      <c r="P35" s="2"/>
     </row>
     <row r="36" spans="2:16">
-      <c r="B36" s="6"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="6"/>
-      <c r="M36" s="6"/>
-      <c r="N36" s="6"/>
-      <c r="O36" s="6"/>
-      <c r="P36" s="6"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
+      <c r="L36" s="2"/>
+      <c r="M36" s="2"/>
+      <c r="N36" s="2"/>
+      <c r="O36" s="2"/>
+      <c r="P36" s="2"/>
     </row>
     <row r="37" spans="2:16">
-      <c r="B37" s="6"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="6"/>
-      <c r="K37" s="6"/>
-      <c r="L37" s="6"/>
-      <c r="M37" s="6"/>
-      <c r="N37" s="6"/>
-      <c r="O37" s="6"/>
-      <c r="P37" s="6"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
+      <c r="L37" s="2"/>
+      <c r="M37" s="2"/>
+      <c r="N37" s="2"/>
+      <c r="O37" s="2"/>
+      <c r="P37" s="2"/>
     </row>
     <row r="38" spans="2:16">
-      <c r="B38" s="6"/>
-      <c r="C38" s="6"/>
-      <c r="D38" s="6"/>
-      <c r="E38" s="6"/>
-      <c r="F38" s="6"/>
-      <c r="G38" s="6"/>
-      <c r="H38" s="6"/>
-      <c r="I38" s="6"/>
-      <c r="J38" s="6"/>
-      <c r="K38" s="6"/>
-      <c r="L38" s="6"/>
-      <c r="M38" s="6"/>
-      <c r="N38" s="6"/>
-      <c r="O38" s="6"/>
-      <c r="P38" s="6"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="2"/>
+      <c r="K38" s="2"/>
+      <c r="L38" s="2"/>
+      <c r="M38" s="2"/>
+      <c r="N38" s="2"/>
+      <c r="O38" s="2"/>
+      <c r="P38" s="2"/>
     </row>
     <row r="39" spans="2:16">
-      <c r="B39" s="6"/>
-      <c r="C39" s="6"/>
-      <c r="D39" s="6"/>
-      <c r="E39" s="6"/>
-      <c r="F39" s="6"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="6"/>
-      <c r="I39" s="6"/>
-      <c r="J39" s="6"/>
-      <c r="K39" s="6"/>
-      <c r="L39" s="6"/>
-      <c r="M39" s="6"/>
-      <c r="N39" s="6"/>
-      <c r="O39" s="6"/>
-      <c r="P39" s="6"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="2"/>
+      <c r="K39" s="2"/>
+      <c r="L39" s="2"/>
+      <c r="M39" s="2"/>
+      <c r="N39" s="2"/>
+      <c r="O39" s="2"/>
+      <c r="P39" s="2"/>
     </row>
     <row r="40" spans="2:16" ht="10" customHeight="1"/>
     <row r="41" spans="2:16" ht="17" customHeight="1">
       <c r="B41" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
@@ -3411,196 +3433,196 @@
       <c r="P41" s="5"/>
     </row>
     <row r="42" spans="2:16">
-      <c r="B42" s="6"/>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="6"/>
-      <c r="F42" s="6"/>
-      <c r="G42" s="6"/>
-      <c r="H42" s="6"/>
-      <c r="I42" s="6"/>
-      <c r="J42" s="6"/>
-      <c r="K42" s="6"/>
-      <c r="L42" s="6"/>
-      <c r="M42" s="6"/>
-      <c r="N42" s="6"/>
-      <c r="O42" s="6"/>
-      <c r="P42" s="6"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+      <c r="I42" s="2"/>
+      <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
+      <c r="L42" s="2"/>
+      <c r="M42" s="2"/>
+      <c r="N42" s="2"/>
+      <c r="O42" s="2"/>
+      <c r="P42" s="2"/>
     </row>
     <row r="43" spans="2:16">
-      <c r="B43" s="6"/>
-      <c r="C43" s="6"/>
-      <c r="D43" s="6"/>
-      <c r="E43" s="6"/>
-      <c r="F43" s="6"/>
-      <c r="G43" s="6"/>
-      <c r="H43" s="6"/>
-      <c r="I43" s="6"/>
-      <c r="J43" s="6"/>
-      <c r="K43" s="6"/>
-      <c r="L43" s="6"/>
-      <c r="M43" s="6"/>
-      <c r="N43" s="6"/>
-      <c r="O43" s="6"/>
-      <c r="P43" s="6"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+      <c r="I43" s="2"/>
+      <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
+      <c r="L43" s="2"/>
+      <c r="M43" s="2"/>
+      <c r="N43" s="2"/>
+      <c r="O43" s="2"/>
+      <c r="P43" s="2"/>
     </row>
     <row r="44" spans="2:16">
-      <c r="B44" s="6"/>
-      <c r="C44" s="6"/>
-      <c r="D44" s="6"/>
-      <c r="E44" s="6"/>
-      <c r="F44" s="6"/>
-      <c r="G44" s="6"/>
-      <c r="H44" s="6"/>
-      <c r="I44" s="6"/>
-      <c r="J44" s="6"/>
-      <c r="K44" s="6"/>
-      <c r="L44" s="6"/>
-      <c r="M44" s="6"/>
-      <c r="N44" s="6"/>
-      <c r="O44" s="6"/>
-      <c r="P44" s="6"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+      <c r="I44" s="2"/>
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
+      <c r="L44" s="2"/>
+      <c r="M44" s="2"/>
+      <c r="N44" s="2"/>
+      <c r="O44" s="2"/>
+      <c r="P44" s="2"/>
     </row>
     <row r="45" spans="2:16">
-      <c r="B45" s="6"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="6"/>
-      <c r="F45" s="6"/>
-      <c r="G45" s="6"/>
-      <c r="H45" s="6"/>
-      <c r="I45" s="6"/>
-      <c r="J45" s="6"/>
-      <c r="K45" s="6"/>
-      <c r="L45" s="6"/>
-      <c r="M45" s="6"/>
-      <c r="N45" s="6"/>
-      <c r="O45" s="6"/>
-      <c r="P45" s="6"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
+      <c r="I45" s="2"/>
+      <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
+      <c r="L45" s="2"/>
+      <c r="M45" s="2"/>
+      <c r="N45" s="2"/>
+      <c r="O45" s="2"/>
+      <c r="P45" s="2"/>
     </row>
     <row r="46" spans="2:16">
-      <c r="B46" s="6"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="6"/>
-      <c r="E46" s="6"/>
-      <c r="F46" s="6"/>
-      <c r="G46" s="6"/>
-      <c r="H46" s="6"/>
-      <c r="I46" s="6"/>
-      <c r="J46" s="6"/>
-      <c r="K46" s="6"/>
-      <c r="L46" s="6"/>
-      <c r="M46" s="6"/>
-      <c r="N46" s="6"/>
-      <c r="O46" s="6"/>
-      <c r="P46" s="6"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+      <c r="G46" s="2"/>
+      <c r="H46" s="2"/>
+      <c r="I46" s="2"/>
+      <c r="J46" s="2"/>
+      <c r="K46" s="2"/>
+      <c r="L46" s="2"/>
+      <c r="M46" s="2"/>
+      <c r="N46" s="2"/>
+      <c r="O46" s="2"/>
+      <c r="P46" s="2"/>
     </row>
     <row r="47" spans="2:16">
-      <c r="B47" s="6"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="6"/>
-      <c r="E47" s="6"/>
-      <c r="F47" s="6"/>
-      <c r="G47" s="6"/>
-      <c r="H47" s="6"/>
-      <c r="I47" s="6"/>
-      <c r="J47" s="6"/>
-      <c r="K47" s="6"/>
-      <c r="L47" s="6"/>
-      <c r="M47" s="6"/>
-      <c r="N47" s="6"/>
-      <c r="O47" s="6"/>
-      <c r="P47" s="6"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2"/>
+      <c r="J47" s="2"/>
+      <c r="K47" s="2"/>
+      <c r="L47" s="2"/>
+      <c r="M47" s="2"/>
+      <c r="N47" s="2"/>
+      <c r="O47" s="2"/>
+      <c r="P47" s="2"/>
     </row>
     <row r="48" spans="2:16">
-      <c r="B48" s="6"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
-      <c r="E48" s="6"/>
-      <c r="F48" s="6"/>
-      <c r="G48" s="6"/>
-      <c r="H48" s="6"/>
-      <c r="I48" s="6"/>
-      <c r="J48" s="6"/>
-      <c r="K48" s="6"/>
-      <c r="L48" s="6"/>
-      <c r="M48" s="6"/>
-      <c r="N48" s="6"/>
-      <c r="O48" s="6"/>
-      <c r="P48" s="6"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="2"/>
+      <c r="J48" s="2"/>
+      <c r="K48" s="2"/>
+      <c r="L48" s="2"/>
+      <c r="M48" s="2"/>
+      <c r="N48" s="2"/>
+      <c r="O48" s="2"/>
+      <c r="P48" s="2"/>
     </row>
     <row r="49" spans="2:16">
-      <c r="B49" s="6"/>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6"/>
-      <c r="E49" s="6"/>
-      <c r="F49" s="6"/>
-      <c r="G49" s="6"/>
-      <c r="H49" s="6"/>
-      <c r="I49" s="6"/>
-      <c r="J49" s="6"/>
-      <c r="K49" s="6"/>
-      <c r="L49" s="6"/>
-      <c r="M49" s="6"/>
-      <c r="N49" s="6"/>
-      <c r="O49" s="6"/>
-      <c r="P49" s="6"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2"/>
+      <c r="H49" s="2"/>
+      <c r="I49" s="2"/>
+      <c r="J49" s="2"/>
+      <c r="K49" s="2"/>
+      <c r="L49" s="2"/>
+      <c r="M49" s="2"/>
+      <c r="N49" s="2"/>
+      <c r="O49" s="2"/>
+      <c r="P49" s="2"/>
     </row>
     <row r="50" spans="2:16">
-      <c r="B50" s="6"/>
-      <c r="C50" s="6"/>
-      <c r="D50" s="6"/>
-      <c r="E50" s="6"/>
-      <c r="F50" s="6"/>
-      <c r="G50" s="6"/>
-      <c r="H50" s="6"/>
-      <c r="I50" s="6"/>
-      <c r="J50" s="6"/>
-      <c r="K50" s="6"/>
-      <c r="L50" s="6"/>
-      <c r="M50" s="6"/>
-      <c r="N50" s="6"/>
-      <c r="O50" s="6"/>
-      <c r="P50" s="6"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
+      <c r="F50" s="2"/>
+      <c r="G50" s="2"/>
+      <c r="H50" s="2"/>
+      <c r="I50" s="2"/>
+      <c r="J50" s="2"/>
+      <c r="K50" s="2"/>
+      <c r="L50" s="2"/>
+      <c r="M50" s="2"/>
+      <c r="N50" s="2"/>
+      <c r="O50" s="2"/>
+      <c r="P50" s="2"/>
     </row>
     <row r="51" spans="2:16">
-      <c r="B51" s="6"/>
-      <c r="C51" s="6"/>
-      <c r="D51" s="6"/>
-      <c r="E51" s="6"/>
-      <c r="F51" s="6"/>
-      <c r="G51" s="6"/>
-      <c r="H51" s="6"/>
-      <c r="I51" s="6"/>
-      <c r="J51" s="6"/>
-      <c r="K51" s="6"/>
-      <c r="L51" s="6"/>
-      <c r="M51" s="6"/>
-      <c r="N51" s="6"/>
-      <c r="O51" s="6"/>
-      <c r="P51" s="6"/>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
+      <c r="I51" s="2"/>
+      <c r="J51" s="2"/>
+      <c r="K51" s="2"/>
+      <c r="L51" s="2"/>
+      <c r="M51" s="2"/>
+      <c r="N51" s="2"/>
+      <c r="O51" s="2"/>
+      <c r="P51" s="2"/>
     </row>
     <row r="52" spans="2:16">
-      <c r="B52" s="6"/>
-      <c r="C52" s="6"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6"/>
-      <c r="F52" s="6"/>
-      <c r="G52" s="6"/>
-      <c r="H52" s="6"/>
-      <c r="I52" s="6"/>
-      <c r="J52" s="6"/>
-      <c r="K52" s="6"/>
-      <c r="L52" s="6"/>
-      <c r="M52" s="6"/>
-      <c r="N52" s="6"/>
-      <c r="O52" s="6"/>
-      <c r="P52" s="6"/>
+      <c r="B52" s="2"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="2"/>
+      <c r="K52" s="2"/>
+      <c r="L52" s="2"/>
+      <c r="M52" s="2"/>
+      <c r="N52" s="2"/>
+      <c r="O52" s="2"/>
+      <c r="P52" s="2"/>
     </row>
     <row r="53" spans="2:16" ht="8" customHeight="1"/>
     <row r="54" spans="2:16" ht="17" customHeight="1">
       <c r="B54" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5"/>
@@ -3618,279 +3640,279 @@
       <c r="P54" s="5"/>
     </row>
     <row r="55" spans="2:16" ht="16" customHeight="1">
-      <c r="B55" s="16"/>
-      <c r="C55" s="16" t="s">
+      <c r="B55" s="15"/>
+      <c r="C55" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="D55" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="D55" s="16" t="s">
+      <c r="E55" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="E55" s="16" t="s">
+      <c r="F55" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="F55" s="16" t="s">
+      <c r="G55" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="G55" s="16" t="s">
+      <c r="H55" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="H55" s="16" t="s">
+      <c r="I55" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="I55" s="16" t="s">
+      <c r="J55" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="J55" s="16" t="s">
+      <c r="K55" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="K55" s="16" t="s">
+      <c r="L55" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="L55" s="16" t="s">
+      <c r="M55" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="M55" s="16" t="s">
+      <c r="N55" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="N55" s="16" t="s">
+      <c r="O55" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="O55" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="P55" s="16"/>
+      <c r="P55" s="15"/>
     </row>
     <row r="56" spans="2:16" ht="14" customHeight="1">
-      <c r="B56" s="17">
+      <c r="B56" s="16">
         <v>2026</v>
       </c>
-      <c r="C56" s="18">
+      <c r="C56" s="17">
         <v>0.68</v>
       </c>
-      <c r="D56" s="18">
+      <c r="D56" s="17">
         <v>1.46</v>
       </c>
-      <c r="E56" s="19"/>
-      <c r="F56" s="19"/>
-      <c r="G56" s="19"/>
-      <c r="H56" s="19"/>
-      <c r="I56" s="19"/>
-      <c r="J56" s="19"/>
-      <c r="K56" s="19"/>
-      <c r="L56" s="19"/>
-      <c r="M56" s="19"/>
-      <c r="N56" s="19"/>
-      <c r="O56" s="20">
+      <c r="E56" s="18"/>
+      <c r="F56" s="18"/>
+      <c r="G56" s="18"/>
+      <c r="H56" s="18"/>
+      <c r="I56" s="18"/>
+      <c r="J56" s="18"/>
+      <c r="K56" s="18"/>
+      <c r="L56" s="18"/>
+      <c r="M56" s="18"/>
+      <c r="N56" s="18"/>
+      <c r="O56" s="19">
         <v>2.15</v>
       </c>
-      <c r="P56" s="20"/>
+      <c r="P56" s="19"/>
     </row>
     <row r="57" spans="2:16" ht="14" customHeight="1">
-      <c r="B57" s="21">
+      <c r="B57" s="20">
         <v>2025</v>
       </c>
-      <c r="C57" s="22">
+      <c r="C57" s="21">
         <v>0.24</v>
       </c>
-      <c r="D57" s="22">
+      <c r="D57" s="21">
         <v>0.6</v>
       </c>
-      <c r="E57" s="22">
+      <c r="E57" s="21">
         <v>0.89</v>
       </c>
-      <c r="F57" s="22">
+      <c r="F57" s="21">
         <v>0.98</v>
       </c>
-      <c r="G57" s="22">
+      <c r="G57" s="21">
         <v>1.48</v>
       </c>
-      <c r="H57" s="22">
+      <c r="H57" s="21">
         <v>4.24</v>
       </c>
-      <c r="I57" s="22">
+      <c r="I57" s="21">
         <v>0.1</v>
       </c>
-      <c r="J57" s="22">
+      <c r="J57" s="21">
         <v>2.41</v>
       </c>
-      <c r="K57" s="22">
+      <c r="K57" s="21">
         <v>0.29</v>
       </c>
-      <c r="L57" s="22">
+      <c r="L57" s="21">
         <v>0.05</v>
       </c>
-      <c r="M57" s="23">
+      <c r="M57" s="22">
         <v>-0.54</v>
       </c>
-      <c r="N57" s="22">
+      <c r="N57" s="21">
         <v>0.38</v>
       </c>
-      <c r="O57" s="24">
+      <c r="O57" s="23">
         <v>11.61</v>
       </c>
-      <c r="P57" s="24"/>
+      <c r="P57" s="23"/>
     </row>
     <row r="58" spans="2:16" ht="14" customHeight="1">
-      <c r="B58" s="17">
+      <c r="B58" s="16">
         <v>2024</v>
       </c>
-      <c r="C58" s="18">
+      <c r="C58" s="17">
         <v>0.67</v>
       </c>
-      <c r="D58" s="18">
+      <c r="D58" s="17">
         <v>1.24</v>
       </c>
-      <c r="E58" s="18">
+      <c r="E58" s="17">
         <v>0.66</v>
       </c>
-      <c r="F58" s="18">
+      <c r="F58" s="17">
         <v>0.86</v>
       </c>
-      <c r="G58" s="18">
+      <c r="G58" s="17">
         <v>5.91</v>
       </c>
-      <c r="H58" s="18">
+      <c r="H58" s="17">
         <v>1.16</v>
       </c>
-      <c r="I58" s="18">
+      <c r="I58" s="17">
         <v>0.24</v>
       </c>
-      <c r="J58" s="18">
+      <c r="J58" s="17">
         <v>2.58</v>
       </c>
-      <c r="K58" s="18">
+      <c r="K58" s="17">
         <v>0.35</v>
       </c>
-      <c r="L58" s="18">
+      <c r="L58" s="17">
         <v>1.12</v>
       </c>
-      <c r="M58" s="18">
+      <c r="M58" s="17">
         <v>4.99</v>
       </c>
-      <c r="N58" s="18">
+      <c r="N58" s="17">
         <v>1.22</v>
       </c>
-      <c r="O58" s="20">
+      <c r="O58" s="19">
         <v>22.93</v>
       </c>
-      <c r="P58" s="20"/>
+      <c r="P58" s="19"/>
     </row>
     <row r="59" spans="2:16" ht="14" customHeight="1">
-      <c r="B59" s="21">
+      <c r="B59" s="20">
         <v>2023</v>
       </c>
-      <c r="C59" s="22">
+      <c r="C59" s="21">
         <v>1.44</v>
       </c>
-      <c r="D59" s="22">
+      <c r="D59" s="21">
         <v>2.62</v>
       </c>
-      <c r="E59" s="22">
+      <c r="E59" s="21">
         <v>2.19</v>
       </c>
-      <c r="F59" s="22">
+      <c r="F59" s="21">
         <v>2.46</v>
       </c>
-      <c r="G59" s="22">
+      <c r="G59" s="21">
         <v>4.32</v>
       </c>
-      <c r="H59" s="22">
+      <c r="H59" s="21">
         <v>2.71</v>
       </c>
-      <c r="I59" s="22">
+      <c r="I59" s="21">
         <v>1.97</v>
       </c>
-      <c r="J59" s="22">
+      <c r="J59" s="21">
         <v>3.56</v>
       </c>
-      <c r="K59" s="22">
+      <c r="K59" s="21">
         <v>0.96</v>
       </c>
-      <c r="L59" s="22">
+      <c r="L59" s="21">
         <v>0.26</v>
       </c>
-      <c r="M59" s="22">
+      <c r="M59" s="21">
         <v>0.93</v>
       </c>
-      <c r="N59" s="22">
+      <c r="N59" s="21">
         <v>0.89</v>
       </c>
-      <c r="O59" s="24">
+      <c r="O59" s="23">
         <v>27.11</v>
       </c>
-      <c r="P59" s="24"/>
+      <c r="P59" s="23"/>
     </row>
     <row r="60" spans="2:16" ht="14" customHeight="1">
-      <c r="B60" s="17">
+      <c r="B60" s="16">
         <v>2022</v>
       </c>
-      <c r="C60" s="19"/>
-      <c r="D60" s="19"/>
-      <c r="E60" s="19"/>
-      <c r="F60" s="19"/>
-      <c r="G60" s="19"/>
-      <c r="H60" s="19"/>
-      <c r="I60" s="18">
+      <c r="C60" s="18"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="18"/>
+      <c r="F60" s="18"/>
+      <c r="G60" s="18"/>
+      <c r="H60" s="18"/>
+      <c r="I60" s="17">
         <v>5.74</v>
       </c>
-      <c r="J60" s="18">
+      <c r="J60" s="17">
         <v>3.29</v>
       </c>
-      <c r="K60" s="18">
+      <c r="K60" s="17">
         <v>2.62</v>
       </c>
-      <c r="L60" s="18">
+      <c r="L60" s="17">
         <v>2.7</v>
       </c>
-      <c r="M60" s="18">
+      <c r="M60" s="17">
         <v>1.66</v>
       </c>
-      <c r="N60" s="18">
+      <c r="N60" s="17">
         <v>1.12</v>
       </c>
-      <c r="O60" s="20">
+      <c r="O60" s="19">
         <v>18.33</v>
       </c>
-      <c r="P60" s="20"/>
+      <c r="P60" s="19"/>
     </row>
     <row r="61" spans="2:16" ht="6" customHeight="1"/>
     <row r="62" spans="2:16" ht="40" customHeight="1">
-      <c r="B62" s="25" t="s">
+      <c r="B62" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="C62" s="24"/>
+      <c r="D62" s="24"/>
+      <c r="E62" s="24"/>
+      <c r="F62" s="24"/>
+      <c r="G62" s="24"/>
+      <c r="H62" s="24"/>
+      <c r="I62" s="24"/>
+      <c r="J62" s="24"/>
+      <c r="K62" s="24"/>
+      <c r="L62" s="24"/>
+      <c r="M62" s="24"/>
+      <c r="N62" s="24"/>
+      <c r="O62" s="24"/>
+      <c r="P62" s="24"/>
+    </row>
+    <row r="63" spans="2:16" ht="16" customHeight="1">
+      <c r="B63" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="C62" s="25"/>
-      <c r="D62" s="25"/>
-      <c r="E62" s="25"/>
-      <c r="F62" s="25"/>
-      <c r="G62" s="25"/>
-      <c r="H62" s="25"/>
-      <c r="I62" s="25"/>
-      <c r="J62" s="25"/>
-      <c r="K62" s="25"/>
-      <c r="L62" s="25"/>
-      <c r="M62" s="25"/>
-      <c r="N62" s="25"/>
-      <c r="O62" s="25"/>
-      <c r="P62" s="25"/>
-    </row>
-    <row r="63" spans="2:16" ht="16" customHeight="1">
-      <c r="B63" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="C63" s="11"/>
-      <c r="D63" s="11"/>
-      <c r="E63" s="11"/>
-      <c r="F63" s="11"/>
-      <c r="G63" s="11"/>
-      <c r="H63" s="11"/>
-      <c r="I63" s="11"/>
-      <c r="J63" s="11"/>
-      <c r="K63" s="11"/>
-      <c r="L63" s="11"/>
-      <c r="M63" s="11"/>
-      <c r="N63" s="11"/>
-      <c r="O63" s="11"/>
-      <c r="P63" s="11"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="10"/>
+      <c r="E63" s="10"/>
+      <c r="F63" s="10"/>
+      <c r="G63" s="10"/>
+      <c r="H63" s="10"/>
+      <c r="I63" s="10"/>
+      <c r="J63" s="10"/>
+      <c r="K63" s="10"/>
+      <c r="L63" s="10"/>
+      <c r="M63" s="10"/>
+      <c r="N63" s="10"/>
+      <c r="O63" s="10"/>
+      <c r="P63" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="107">

</xml_diff>